<commit_message>
docs: record Android CLI public chat test
</commit_message>
<xml_diff>
--- a/bitchat-cli-feature-tracker.xlsx
+++ b/bitchat-cli-feature-tracker.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Features'!$A$1:$H$59</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Errors'!$A$1:$H$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Errors'!$A$1:$H$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2773,17 +2773,17 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>tests/test_app.py; tests/test_transport.py</t>
+          <t>tests/test_app.py; tests/test_transport.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>Android package com.bitchat.droid</t>
+          <t>Android package com.bitchat.droid; Android_to_cli_1900; cli_to_android_1921</t>
         </is>
       </c>
     </row>
@@ -3188,7 +3188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3327,8 +3327,50 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>ERR-003</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Test procedure</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>The first inbox query ran before the asynchronous Android write had been persisted.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>The message was temporarily absent from the CLI query even though it arrived moments later.</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Test procedure</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>messages.jsonl and daemon.log show Android_to_cli_1900 at 18:19:57/18:21:00</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Wait for delivery or poll with a bounded timeout before declaring a delivery failure.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H3"/>
+  <autoFilter ref="A1:H4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record Android CLI DM test
</commit_message>
<xml_diff>
--- a/bitchat-cli-feature-tracker.xlsx
+++ b/bitchat-cli-feature-tracker.xlsx
@@ -2815,17 +2815,17 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>tests/test_noise.py; tests/test_transport.py</t>
+          <t>tests/test_noise.py; tests/test_transport.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>Android upstream protocol</t>
+          <t>dm_cli_to_android_1926; Android_to_cli_dm_1927; Android package com.bitchat.droid</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: record Android CLI file test
</commit_message>
<xml_diff>
--- a/bitchat-cli-feature-tracker.xlsx
+++ b/bitchat-cli-feature-tracker.xlsx
@@ -2857,17 +2857,17 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>tests/test_fragments.py; tests/test_transport.py</t>
+          <t>tests/test_fragments.py; tests/test_transport.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>Android upstream file TLV</t>
+          <t>bitchat-test-file.txt; Android photo img_1785004221247.jpg; Android package com.bitchat.droid</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: record reconnect sync test
</commit_message>
<xml_diff>
--- a/bitchat-cli-feature-tracker.xlsx
+++ b/bitchat-cli-feature-tracker.xlsx
@@ -2899,17 +2899,17 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>tests/test_sync.py; tests/test_transport.py</t>
+          <t>tests/test_sync.py; tests/test_transport.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>Android/iOS sync behavior</t>
+          <t>Sync_gap_android_1934 recovered after daemon restart; messages.jsonl count=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: record Nostr fallback blocker
</commit_message>
<xml_diff>
--- a/bitchat-cli-feature-tracker.xlsx
+++ b/bitchat-cli-feature-tracker.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Features'!$A$1:$H$59</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Errors'!$A$1:$H$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Errors'!$A$1:$H$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2941,17 +2941,17 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>tests/test_nostr.py; src/bitchat_cli/app.py</t>
+          <t>tests/test_nostr.py; src/bitchat_cli/app.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>CLI routed nostr_fallback_cli_1938 via Nostr; Android UI did not surface it during bounded observation</t>
         </is>
       </c>
     </row>
@@ -3188,7 +3188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3369,8 +3369,50 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>ERR-004</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Nostr fallback</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>The CLI returned via nostr [nostr_fallback] and persisted nostr_fallback_cli_1938, but the Android UI did not show the DM during the bounded observation window.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Offline cross-platform DM delivery is not confirmed; BLE behavior remains unaffected.</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>messages.jsonl message_id nostr-1785004686603; Android UI/logcat; relay availability warnings</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Compare Android Nostr subscription/identity handling with upstream and repeat with a known-current npub.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H4"/>
+  <autoFilter ref="A1:H5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record CLI command smoke tests
</commit_message>
<xml_diff>
--- a/bitchat-cli-feature-tracker.xlsx
+++ b/bitchat-cli-feature-tracker.xlsx
@@ -547,17 +547,17 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>tests/test_app.py; src/bitchat_cli/app.py</t>
+          <t>tests/test_app.py; src/bitchat_cli/app.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>doctor --json returned daemon, scope, and network sections</t>
         </is>
       </c>
     </row>
@@ -925,17 +925,17 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>tests/test_app.py; src/bitchat_cli/app.py</t>
+          <t>tests/test_app.py; src/bitchat_cli/app.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>daemon start returned pid/log/socket paths</t>
         </is>
       </c>
     </row>
@@ -967,17 +967,17 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>src/bitchat_cli/app.py</t>
+          <t>src/bitchat_cli/app.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>daemon status displayed pid, links, peers, advertising, relays, proxy, and watches</t>
         </is>
       </c>
     </row>
@@ -1009,17 +1009,17 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>src/bitchat_cli/app.py</t>
+          <t>src/bitchat_cli/app.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>daemon stop returned clean shutdown for test restarts</t>
         </is>
       </c>
     </row>
@@ -1051,17 +1051,17 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>src/bitchat_cli/queries.py; src/bitchat_cli/app.py</t>
+          <t>src/bitchat_cli/queries.py; src/bitchat_cli/app.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>inbox --json --tail 3 returned persisted public messages</t>
         </is>
       </c>
     </row>
@@ -1135,17 +1135,17 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>src/bitchat_cli/queries.py</t>
+          <t>src/bitchat_cli/queries.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>mesh inbox --json --tail 3 matched public inbox</t>
         </is>
       </c>
     </row>
@@ -1177,17 +1177,17 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>src/bitchat_cli/app.py; src/bitchat_cli/queries.py</t>
+          <t>src/bitchat_cli/app.py; src/bitchat_cli/queries.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>peers --json returned signed peer records and addresses</t>
         </is>
       </c>
     </row>
@@ -1303,17 +1303,17 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>tests/test_app.py; src/bitchat_cli/app.py</t>
+          <t>tests/test_app.py; src/bitchat_cli/app.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>dm_cli_to_android_1926 delivered via BLE</t>
         </is>
       </c>
     </row>
@@ -1345,17 +1345,17 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>tests/test_transport.py; src/bitchat_cli/files.py</t>
+          <t>tests/test_transport.py; src/bitchat_cli/files.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>bitchat-test-file.txt delivered to Android with name/size/MIME</t>
         </is>
       </c>
     </row>
@@ -1387,17 +1387,17 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>src/bitchat_cli/queries.py</t>
+          <t>src/bitchat_cli/queries.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>dm inbox --json returned trueanon conversation preview</t>
         </is>
       </c>
     </row>
@@ -1429,17 +1429,17 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>src/bitchat_cli/queries.py</t>
+          <t>src/bitchat_cli/queries.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>dm history @trueanon --json returned both directions and attachments</t>
         </is>
       </c>
     </row>
@@ -2185,17 +2185,17 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>src/bitchat_cli/social.py; src/bitchat_cli/app.py</t>
+          <t>src/bitchat_cli/social.py; src/bitchat_cli/app.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>social list --json returned linked peers and trust flags</t>
         </is>
       </c>
     </row>
@@ -2269,17 +2269,17 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>src/bitchat_cli/social.py</t>
+          <t>src/bitchat_cli/social.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>favorite then unfavorite toggled trueanon and restored false</t>
         </is>
       </c>
     </row>
@@ -2437,17 +2437,17 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>tests/test_nostr.py; src/bitchat_cli/network.py</t>
+          <t>tests/test_nostr.py; src/bitchat_cli/network.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>network proxy status --json returned disabled/require policy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: record social and geochat state tests
</commit_message>
<xml_diff>
--- a/bitchat-cli-feature-tracker.xlsx
+++ b/bitchat-cli-feature-tracker.xlsx
@@ -1765,17 +1765,17 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>src/bitchat_cli/app.py; src/bitchat_cli/state.py</t>
+          <t>src/bitchat_cli/app.py; src/bitchat_cli/state.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>ezjmgt set with name/note/bookmark/select/teleport, then flags restored</t>
         </is>
       </c>
     </row>
@@ -1807,17 +1807,17 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>src/bitchat_cli/app.py</t>
+          <t>src/bitchat_cli/app.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>geo channel show ezjmgt --json returned metadata and activity counters</t>
         </is>
       </c>
     </row>
@@ -1849,17 +1849,17 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>src/bitchat_cli/app.py</t>
+          <t>src/bitchat_cli/app.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>geo channel list --bookmarked --json filtered bookmarked channels</t>
         </is>
       </c>
     </row>
@@ -1975,17 +1975,17 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>src/bitchat_cli/app.py; src/bitchat_cli/queries.py</t>
+          <t>src/bitchat_cli/app.py; src/bitchat_cli/queries.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>participant show 6vjvfvy d2df184a675345d8 returned trust state</t>
         </is>
       </c>
     </row>
@@ -2017,17 +2017,17 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>src/bitchat_cli/app.py</t>
+          <t>src/bitchat_cli/app.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>trueanon geochat block then unblock restored neutral state</t>
         </is>
       </c>
     </row>
@@ -2143,17 +2143,17 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>tests/test_geochat.py; src/bitchat_cli/app.py</t>
+          <t>tests/test_geochat.py; src/bitchat_cli/app.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>ezjmgt add/list/remove completed; original watches restored</t>
         </is>
       </c>
     </row>
@@ -2227,17 +2227,17 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>src/bitchat_cli/social.py</t>
+          <t>src/bitchat_cli/social.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>trueanon unlink then relink restored original npub mapping</t>
         </is>
       </c>
     </row>
@@ -2311,17 +2311,17 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>src/bitchat_cli/social.py; src/bitchat_cli/app.py</t>
+          <t>src/bitchat_cli/social.py; src/bitchat_cli/app.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>trueanon block then unblock restored neutral state</t>
         </is>
       </c>
     </row>
@@ -2353,17 +2353,17 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>src/bitchat_cli/verification.py; src/bitchat_cli/app.py</t>
+          <t>src/bitchat_cli/verification.py; src/bitchat_cli/app.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>social fingerprint @trueanon returned noise/signing/verification material</t>
         </is>
       </c>
     </row>
@@ -2479,17 +2479,17 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>tests/test_nostr.py; src/bitchat_cli/network.py</t>
+          <t>tests/test_nostr.py; src/bitchat_cli/network.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>proxy set system --policy prefer then disable restored disabled mode</t>
         </is>
       </c>
     </row>
@@ -2521,17 +2521,17 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>src/bitchat_cli/network.py; src/bitchat_cli/app.py</t>
+          <t>src/bitchat_cli/network.py; src/bitchat_cli/app.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>network proxy test --json returned system policy result</t>
         </is>
       </c>
     </row>
@@ -2563,17 +2563,17 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>src/bitchat_cli/app.py; src/bitchat_cli/state.py</t>
+          <t>src/bitchat_cli/app.py; src/bitchat_cli/state.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>#manual-test join then leave completed</t>
         </is>
       </c>
     </row>
@@ -2605,17 +2605,17 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>src/bitchat_cli/app.py</t>
+          <t>src/bitchat_cli/app.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>topic list --json returned temporary topic flags</t>
         </is>
       </c>
     </row>
@@ -2647,17 +2647,17 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>src/bitchat_cli/app.py; src/bitchat_cli/state.py</t>
+          <t>src/bitchat_cli/app.py; src/bitchat_cli/state.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>#manual-test password set/cleared and retention on/off completed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: record interactive chat and mesh tests
</commit_message>
<xml_diff>
--- a/bitchat-cli-feature-tracker.xlsx
+++ b/bitchat-cli-feature-tracker.xlsx
@@ -589,17 +589,17 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>tests/test_app.py; src/bitchat_cli/app.py</t>
+          <t>tests/test_app.py; src/bitchat_cli/app.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>interactive chat session started, accepted commands, and exited cleanly</t>
         </is>
       </c>
     </row>
@@ -631,17 +631,17 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>tests/test_app.py; tests/test_transport.py</t>
+          <t>tests/test_app.py; tests/test_transport.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>chat_public_1956 plus Android↔CLI public chat evidence</t>
         </is>
       </c>
     </row>
@@ -673,17 +673,17 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>src/bitchat_cli/app.py</t>
+          <t>src/bitchat_cli/app.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>/help printed all documented slash commands</t>
         </is>
       </c>
     </row>
@@ -715,17 +715,17 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>tests/test_transport.py; src/bitchat_cli/transport.py</t>
+          <t>tests/test_transport.py; src/bitchat_cli/transport.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>/name clanker-temp updated then restored clanker</t>
         </is>
       </c>
     </row>
@@ -757,17 +757,17 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>src/bitchat_cli/app.py</t>
+          <t>src/bitchat_cli/app.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>/who listed trueanon and peer ID</t>
         </is>
       </c>
     </row>
@@ -799,17 +799,17 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>tests/test_transport.py; src/bitchat_cli/transport.py</t>
+          <t>tests/test_transport.py; src/bitchat_cli/transport.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>chat_dm_1955 received delivered receipt from trueanon</t>
         </is>
       </c>
     </row>
@@ -841,17 +841,17 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>src/bitchat_cli/app.py</t>
+          <t>src/bitchat_cli/app.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>/clear emitted terminal clear sequence</t>
         </is>
       </c>
     </row>
@@ -883,17 +883,17 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>tests/test_transport.py; src/bitchat_cli/app.py</t>
+          <t>tests/test_transport.py; src/bitchat_cli/app.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>/quit ended the interactive process and daemon restarted cleanly</t>
         </is>
       </c>
     </row>
@@ -1093,17 +1093,17 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>src/bitchat_cli/app.py</t>
+          <t>src/bitchat_cli/app.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>mesh_public_1959 rendered in Android #mesh</t>
         </is>
       </c>
     </row>
@@ -1219,17 +1219,17 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>tests/test_transport.py; src/bitchat_cli/files.py</t>
+          <t>tests/test_transport.py; src/bitchat_cli/files.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>send-file rendered TXT card on Android with 29 B</t>
         </is>
       </c>
     </row>
@@ -1261,17 +1261,17 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>src/bitchat_cli/app.py; src/bitchat_cli/files.py</t>
+          <t>src/bitchat_cli/app.py; src/bitchat_cli/files.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>mesh send-file rendered second TXT card on Android with 29 B</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: record geochat read tests
</commit_message>
<xml_diff>
--- a/bitchat-cli-feature-tracker.xlsx
+++ b/bitchat-cli-feature-tracker.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Features'!$A$1:$H$59</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Errors'!$A$1:$H$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Errors'!$A$1:$H$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1513,17 +1513,17 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>tests/test_geochat.py; src/bitchat_cli/queries.py</t>
+          <t>tests/test_geochat.py; src/bitchat_cli/queries.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>geo inbox 6vjvfv --json returned deduplicated geohash events</t>
         </is>
       </c>
     </row>
@@ -1555,17 +1555,17 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>src/bitchat_cli/queries.py</t>
+          <t>src/bitchat_cli/queries.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>geo who 6vjvfv --json returned an empty current participant list</t>
         </is>
       </c>
     </row>
@@ -1723,17 +1723,17 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>src/bitchat_cli/geochat.py; src/bitchat_cli/app.py</t>
+          <t>src/bitchat_cli/geochat.py; src/bitchat_cli/app.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>lookup stopped because proxy policy=require while proxy mode=disabled</t>
         </is>
       </c>
     </row>
@@ -2101,17 +2101,17 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>src/bitchat_cli/app.py; src/bitchat_cli/queries.py</t>
+          <t>src/bitchat_cli/app.py; src/bitchat_cli/queries.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>geo dm history 6vjvfv @trueanon --json executed with empty history</t>
         </is>
       </c>
     </row>
@@ -3188,7 +3188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3411,8 +3411,50 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>ERR-005</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Geo lookup</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Place lookup refused to run because proxy policy is require while proxy mode is disabled.</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Third-party geocoding is unavailable until a compliant proxy is configured.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Configuration blocker</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>geo lookup Lisbon, Portugal --json</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Configure an approved system/Tor proxy, then rerun lookup.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H5"/>
+  <autoFilter ref="A1:H6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record geo lookup and verification tests
</commit_message>
<xml_diff>
--- a/bitchat-cli-feature-tracker.xlsx
+++ b/bitchat-cli-feature-tracker.xlsx
@@ -1723,7 +1723,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>lookup stopped because proxy policy=require while proxy mode=disabled</t>
+          <t>Lisbon, Portugal lookup returned labels, coordinates, addresses, and geohash levels with system proxy</t>
         </is>
       </c>
     </row>
@@ -2395,17 +2395,17 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Not tested</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>tests/test_noise.py; src/bitchat_cli/verification.py</t>
+          <t>tests/test_noise.py; src/bitchat_cli/verification.py; manual 2026-07-25</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>invalid payload rejected; verify without payload then unverify restored original state</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: refine Nostr fallback test evidence
</commit_message>
<xml_diff>
--- a/bitchat-cli-feature-tracker.xlsx
+++ b/bitchat-cli-feature-tracker.xlsx
@@ -2951,7 +2951,7 @@
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>CLI routed nostr_fallback_cli_1938 via Nostr; Android UI did not surface it during bounded observation</t>
+          <t>CLI published nostr_mutual_favorite_direct after both sides were favorited; Android 1.7.4 still had no DM Nostr subscription and did not surface it</t>
         </is>
       </c>
     </row>
@@ -3387,7 +3387,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>The CLI returned via nostr [nostr_fallback] and persisted nostr_fallback_cli_1938, but the Android UI did not show the DM during the bounded observation window.</t>
+          <t>The CLI published nostr_mutual_favorite_direct after both sides were favorited, but Android 1.7.4 still had no DM Nostr subscription and did not show the message.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -3397,17 +3397,17 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Configuration blocker</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>messages.jsonl message_id nostr-1785004686603; Android UI/logcat; relay availability warnings</t>
+          <t>Android UI marked clanker as an offline favorite; logcat showed only location-notes subscriptions and no DM subscription</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Compare Android Nostr subscription/identity handling with upstream and repeat with a known-current npub.</t>
+          <t>Configure/verify the Android Nostr identity and mutual-favorite DM subscription, then repeat with a known-current npub.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test: record geo story outcomes
</commit_message>
<xml_diff>
--- a/bitchat-cli-feature-tracker.xlsx
+++ b/bitchat-cli-feature-tracker.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="Rcb9bee3dcfc049ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R9211f7c38a9246e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Errors" sheetId="3" r:id="R46d2d4aae24d424d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="Rafa3909e82d04783"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R2f60dd77e0e3458c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Errors" sheetId="3" r:id="R167944e7b3ee4662"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1384,20 +1384,16 @@
           <x:t xml:space="preserve">Publishes a signed kind 20000 event with optional PoW, teleport, and privacy acknowledgement.</x:t>
         </x:is>
       </x:c>
-      <x:c r="F24" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not tested</x:t>
-        </x:is>
+      <x:c r="F24" s="2" t="str">
+        <x:v>Blocked</x:v>
       </x:c>
       <x:c r="G24" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">tests/test_geochat.py; src/bitchat_cli/app.py</x:t>
         </x:is>
       </x:c>
-      <x:c r="H24" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">README.md</x:t>
-        </x:is>
+      <x:c r="H24" s="2" t="str">
+        <x:v>geo send 6vjvfv manual_geo_send_test_20260725 reached the relay but received HTTP 503; a real-location retry at #etgcx was not authorized</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -1804,20 +1800,16 @@
           <x:t xml:space="preserve">Publishes a persistent kind 1 note at building precision.</x:t>
         </x:is>
       </x:c>
-      <x:c r="F34" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not tested</x:t>
-        </x:is>
+      <x:c r="F34" s="2" t="str">
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="G34" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">tests/test_geochat.py; src/bitchat_cli/location_notes.py</x:t>
         </x:is>
       </x:c>
-      <x:c r="H34" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">README.md</x:t>
-        </x:is>
+      <x:c r="H34" s="2" t="str">
+        <x:v>published manual_location_note_test_20260725 at u4pruyd8 with event id 0c76de538ed30911f55d9b1c37493653ffa395ab4316533a507237722e34cce0</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -1846,20 +1838,16 @@
           <x:t xml:space="preserve">Fetches and limits persistent notes for one building geohash.</x:t>
         </x:is>
       </x:c>
-      <x:c r="F35" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not tested</x:t>
-        </x:is>
+      <x:c r="F35" s="2" t="str">
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="G35" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">src/bitchat_cli/location_notes.py</x:t>
         </x:is>
       </x:c>
-      <x:c r="H35" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">README.md</x:t>
-        </x:is>
+      <x:c r="H35" s="2" t="str">
+        <x:v>geo notes list u4pruyd8 --json returned the published event, content, geohash, and nickname clanker</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -1972,20 +1960,16 @@
           <x:t xml:space="preserve">Uses the deterministic per-geohash identity and embedded BitChat payload.</x:t>
         </x:is>
       </x:c>
-      <x:c r="F38" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Not tested</x:t>
-        </x:is>
+      <x:c r="F38" s="2" t="str">
+        <x:v>Blocked</x:v>
       </x:c>
       <x:c r="G38" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">tests/test_geochat.py; src/bitchat_cli/app.py</x:t>
         </x:is>
       </x:c>
-      <x:c r="H38" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">README.md</x:t>
-        </x:is>
+      <x:c r="H38" s="2" t="str">
+        <x:v>geo dm send 6vjvfv @anon4708 queued geo-dm-1785014611130 but history stayed empty; retry at real phone channel #etgcx requires explicit location-payload approval</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -2935,7 +2919,7 @@
       </x:c>
       <x:c r="B3" s="2" t="n">
         <x:f>COUNTIF(Features!F2:F59,"Passed")</x:f>
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C3" s="2" t="inlineStr">
         <x:is>
@@ -2967,7 +2951,7 @@
       </x:c>
       <x:c r="B5" s="2" t="n">
         <x:f>COUNTIF(Features!F2:F59,"Blocked")</x:f>
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C5" s="2" t="inlineStr">
         <x:is>
@@ -2983,7 +2967,7 @@
       </x:c>
       <x:c r="B6" s="2" t="n">
         <x:f>COUNTIF(Features!F2:F59,"Not tested")</x:f>
-        <x:v>4</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C6" s="2" t="inlineStr">
         <x:is>
@@ -2999,7 +2983,7 @@
       </x:c>
       <x:c r="B7" s="4" t="n">
         <x:f>IFERROR(B3/B2,0)</x:f>
-        <x:v>0.9137931034482759</x:v>
+        <x:v>0.9482758620689655</x:v>
       </x:c>
       <x:c r="C7" s="2" t="inlineStr">
         <x:is>
@@ -3377,6 +3361,32 @@
         <x:v>Clarify the supported scope or implement named-channel parity only as a port of the upstream behavior; do not present local metadata as remote membership.</x:v>
       </x:c>
     </x:row>
+    <x:row r="8" ht="72" customHeight="1">
+      <x:c r="A8" s="6" t="str">
+        <x:v>ERR-007</x:v>
+      </x:c>
+      <x:c r="B8" s="6" t="str">
+        <x:v>2026-07-25</x:v>
+      </x:c>
+      <x:c r="C8" s="6" t="str">
+        <x:v>Geo DM</x:v>
+      </x:c>
+      <x:c r="D8" s="6" t="str">
+        <x:v>A synthetic geo DM was queued for 6vjvfv but the recipient history remained empty; the actual phone channel is #etgcx in Funchal.</x:v>
+      </x:c>
+      <x:c r="E8" s="6" t="str">
+        <x:v>Geo DM delivery is not confirmed, and a real-location retry needs explicit approval for publishing to the phone's geohash.</x:v>
+      </x:c>
+      <x:c r="F8" s="6" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="G8" s="6" t="str">
+        <x:v>geo dm send 6vjvfv @anon4708 manual_geo_dm_test_20260725; geo dm history 6vjvfv anon4708 --json returned []</x:v>
+      </x:c>
+      <x:c r="H8" s="6" t="str">
+        <x:v>Obtain explicit approval for the exact #etgcx payload, then verify receipt on Android and in the CLI history.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: close geochat verification procedure
</commit_message>
<xml_diff>
--- a/bitchat-cli-feature-tracker.xlsx
+++ b/bitchat-cli-feature-tracker.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="Rafa3909e82d04783"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R2f60dd77e0e3458c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Errors" sheetId="3" r:id="R167944e7b3ee4662"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="R96d93a2277594b59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R525ffa6d33174e1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Errors" sheetId="3" r:id="Rfe128f5fcfcf4228"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3235,20 +3235,14 @@
           <x:t xml:space="preserve">The message was temporarily absent from the CLI query even though it arrived moments later.</x:t>
         </x:is>
       </x:c>
-      <x:c r="F4" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Test procedure</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G4" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">messages.jsonl and daemon.log show Android_to_cli_1900 at 18:19:57/18:21:00</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H4" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Wait for delivery or poll with a bounded timeout before declaring a delivery failure.</x:t>
-        </x:is>
+      <x:c r="F4" s="2" t="str">
+        <x:v>Fixed</x:v>
+      </x:c>
+      <x:c r="G4" s="2" t="str">
+        <x:v>ca5645c; README.md manual geochat verification now requires the same device geohash and explicit inbox/history confirmation</x:v>
+      </x:c>
+      <x:c r="H4" s="2" t="str">
+        <x:v>Use the documented same-geohash verification procedure and do not treat a queued event as delivered.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">

</xml_diff>

<commit_message>
test: record repeated relay failure
</commit_message>
<xml_diff>
--- a/bitchat-cli-feature-tracker.xlsx
+++ b/bitchat-cli-feature-tracker.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="R96d93a2277594b59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R525ffa6d33174e1e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Errors" sheetId="3" r:id="Rfe128f5fcfcf4228"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="R74baf60c2f6a487d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R548315705e47412c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Errors" sheetId="3" r:id="R79c10c1ec96d4d85"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1393,7 +1393,7 @@
         </x:is>
       </x:c>
       <x:c r="H24" s="2" t="str">
-        <x:v>geo send 6vjvfv manual_geo_send_test_20260725 reached the relay but received HTTP 503; a real-location retry at #etgcx was not authorized</x:v>
+        <x:v>repeated geo send 6vjvfv manual_geo_send_test_20260725 attempts were rejected with HTTP 503; a real-location retry at #etgcx was not authorized</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -3156,10 +3156,8 @@
           <x:t xml:space="preserve">External dependency</x:t>
         </x:is>
       </x:c>
-      <x:c r="G2" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">daemon.log during manual test</x:t>
-        </x:is>
+      <x:c r="G2" s="2" t="str">
+        <x:v>daemon.log during manual test; repeated geo send 6vjvfv manual_geo_send_test_20260725 attempts returned HTTP 503</x:v>
       </x:c>
       <x:c r="H2" s="2" t="inlineStr">
         <x:is>

</xml_diff>

<commit_message>
test: record post-fix command checks
</commit_message>
<xml_diff>
--- a/bitchat-cli-feature-tracker.xlsx
+++ b/bitchat-cli-feature-tracker.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="R74baf60c2f6a487d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R548315705e47412c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Errors" sheetId="3" r:id="R79c10c1ec96d4d85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="R139c6b815ad3402c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R013be087c12e4312"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Errors" sheetId="3" r:id="Rb1b6673a750041d5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -470,10 +470,8 @@
           <x:t xml:space="preserve">tests/test_app.py; src/bitchat_cli/app.py; manual 2026-07-25</x:t>
         </x:is>
       </x:c>
-      <x:c r="H2" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">doctor --json returned daemon, scope, and network sections</x:t>
-        </x:is>
+      <x:c r="H2" s="2" t="str">
+        <x:v>doctor --json returned daemon, scope, and network sections; 70/70 public command --help smoke checks passed</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2344,10 +2342,8 @@
           <x:t xml:space="preserve">tests/test_nostr.py; src/bitchat_cli/network.py; manual 2026-07-25</x:t>
         </x:is>
       </x:c>
-      <x:c r="H47" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">network proxy status --json returned disabled/require policy</x:t>
-        </x:is>
+      <x:c r="H47" s="2" t="str">
+        <x:v>post-fix network proxy status --json returned disabled/require policy</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -2428,10 +2424,8 @@
           <x:t xml:space="preserve">src/bitchat_cli/network.py; src/bitchat_cli/app.py; manual 2026-07-25</x:t>
         </x:is>
       </x:c>
-      <x:c r="H49" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">network proxy test --json returned system policy result</x:t>
-        </x:is>
+      <x:c r="H49" s="2" t="str">
+        <x:v>post-fix network proxy test --json returned healthy=false under disabled/require, confirming fail-closed behavior</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -2590,10 +2584,8 @@
           <x:t xml:space="preserve">tests/; src/bitchat_cli/app.py</x:t>
         </x:is>
       </x:c>
-      <x:c r="H53" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">README.md</x:t>
-        </x:is>
+      <x:c r="H53" s="2" t="str">
+        <x:v>post-fix selftest ok; full pytest regression 176 passed</x:v>
       </x:c>
     </x:row>
     <x:row r="54">

</xml_diff>

<commit_message>
test: isolate relay failure from proxy policy
</commit_message>
<xml_diff>
--- a/bitchat-cli-feature-tracker.xlsx
+++ b/bitchat-cli-feature-tracker.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="R139c6b815ad3402c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R013be087c12e4312"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Errors" sheetId="3" r:id="Rb1b6673a750041d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="R275e1dd301ee49d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R2c9a1eb5578d4380"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Errors" sheetId="3" r:id="Rc11b40e7a8b645eb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1391,7 +1391,7 @@
         </x:is>
       </x:c>
       <x:c r="H24" s="2" t="str">
-        <x:v>repeated geo send 6vjvfv manual_geo_send_test_20260725 attempts were rejected with HTTP 503; a real-location retry at #etgcx was not authorized</x:v>
+        <x:v>repeated geo send 6vjvfv manual_geo_send_test_20260725 attempts were rejected with HTTP 503 under both disabled/require and system/prefer; a real-location retry at #etgcx was not authorized</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -3149,7 +3149,7 @@
         </x:is>
       </x:c>
       <x:c r="G2" s="2" t="str">
-        <x:v>daemon.log during manual test; repeated geo send 6vjvfv manual_geo_send_test_20260725 attempts returned HTTP 503</x:v>
+        <x:v>daemon.log during manual test; repeated geo send 6vjvfv manual_geo_send_test_20260725 attempts returned HTTP 503 under disabled/require and system/prefer</x:v>
       </x:c>
       <x:c r="H2" s="2" t="inlineStr">
         <x:is>

</xml_diff>

<commit_message>
test: refresh regression evidence
</commit_message>
<xml_diff>
--- a/bitchat-cli-feature-tracker.xlsx
+++ b/bitchat-cli-feature-tracker.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="R275e1dd301ee49d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R2c9a1eb5578d4380"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Errors" sheetId="3" r:id="Rc11b40e7a8b645eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="Rb128977f83ee4ed0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R3e990be850194230"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Errors" sheetId="3" r:id="R91310b12593f43ef"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2585,7 +2585,7 @@
         </x:is>
       </x:c>
       <x:c r="H53" s="2" t="str">
-        <x:v>post-fix selftest ok; full pytest regression 176 passed</x:v>
+        <x:v>post-fix selftest ok; full pytest regression 177 passed</x:v>
       </x:c>
     </x:row>
     <x:row r="54">

</xml_diff>

<commit_message>
docs: refresh post-fix manual evidence
</commit_message>
<xml_diff>
--- a/bitchat-cli-feature-tracker.xlsx
+++ b/bitchat-cli-feature-tracker.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="Rb128977f83ee4ed0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R3e990be850194230"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Errors" sheetId="3" r:id="R91310b12593f43ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="R3ed4cc4bab98489b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R7fe467cca1b54c9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Errors" sheetId="3" r:id="R5daaff4de26e4d1f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2624,10 +2624,8 @@
           <x:t xml:space="preserve">20d5577; tests/test_transport.py; src/bitchat_cli/transport.py</x:t>
         </x:is>
       </x:c>
-      <x:c r="H54" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Android upstream: BluetoothMeshService.kt; iOS upstream: BLEService.swift</x:t>
-        </x:is>
+      <x:c r="H54" s="2" t="str">
+        <x:v>post-fix Android room #mesh still displayed &lt;@clanker&gt; cable_public_roundtrip_20260725; peer list later showed clanker as Direct Bluetooth</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
@@ -2666,10 +2664,8 @@
           <x:t xml:space="preserve">tests/test_app.py; tests/test_transport.py; manual 2026-07-25</x:t>
         </x:is>
       </x:c>
-      <x:c r="H55" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Android package com.bitchat.droid; Android_to_cli_1900; cli_to_android_1921</x:t>
-        </x:is>
+      <x:c r="H55" s="2" t="str">
+        <x:v>post-fix CLI→Android cable_public_roundtrip_20260725 was shown in Android #mesh; previous Android→CLI public message Android_to_cli_1900 was persisted</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -2708,10 +2704,8 @@
           <x:t xml:space="preserve">tests/test_noise.py; tests/test_transport.py; manual 2026-07-25</x:t>
         </x:is>
       </x:c>
-      <x:c r="H56" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">dm_cli_to_android_1926; Android_to_cli_dm_1927; Android package com.bitchat.droid</x:t>
-        </x:is>
+      <x:c r="H56" s="2" t="str">
+        <x:v>post-fix CLI→Android postfix_fresh_dm_20260725 appeared in the encrypted direct conversation and CLI history received delivered receipt; Android→CLI Android_to_cli_dm_cable_20260725 was persisted</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
@@ -2750,10 +2744,8 @@
           <x:t xml:space="preserve">tests/test_fragments.py; tests/test_transport.py; manual 2026-07-25</x:t>
         </x:is>
       </x:c>
-      <x:c r="H57" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">bitchat-test-file.txt; Android photo img_1785004221247.jpg; Android package com.bitchat.droid</x:t>
-        </x:is>
+      <x:c r="H57" s="2" t="str">
+        <x:v>previous post-fix manual BLE file roundtrip passed: bitchat-test-file.txt and Android photo persisted with correct metadata</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
@@ -2792,10 +2784,8 @@
           <x:t xml:space="preserve">tests/test_sync.py; tests/test_transport.py; manual 2026-07-25</x:t>
         </x:is>
       </x:c>
-      <x:c r="H58" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Sync_gap_android_1934 recovered after daemon restart; messages.jsonl count=1</x:t>
-        </x:is>
+      <x:c r="H58" s="2" t="str">
+        <x:v>previous post-fix reconnect test recovered Sync_gap_android_1934 once with messages.jsonl count=1</x:v>
       </x:c>
     </x:row>
     <x:row r="59">

</xml_diff>

<commit_message>
docs: record geo dm history fix
</commit_message>
<xml_diff>
--- a/bitchat-cli-feature-tracker.xlsx
+++ b/bitchat-cli-feature-tracker.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="R3ed4cc4bab98489b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R7fe467cca1b54c9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Errors" sheetId="3" r:id="R5daaff4de26e4d1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="Rfeeaba20aa9e499a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Rac45f7e093e54f99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Errors" sheetId="3" r:id="Ra102cdb5d1554d79"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1391,7 +1391,7 @@
         </x:is>
       </x:c>
       <x:c r="H24" s="2" t="str">
-        <x:v>repeated geo send 6vjvfv manual_geo_send_test_20260725 attempts were rejected with HTTP 503 under both disabled/require and system/prefer; a real-location retry at #etgcx was not authorized</x:v>
+        <x:v>geo send 6vjvfv remained blocked by relay HTTP 503; synthetic u4pruyd8 send recheck_geo_send_20260725 queued and was persisted, but no remote inbox confirmation was available</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -1959,7 +1959,7 @@
         </x:is>
       </x:c>
       <x:c r="F38" s="2" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="G38" s="2" t="inlineStr">
         <x:is>
@@ -1967,7 +1967,7 @@
         </x:is>
       </x:c>
       <x:c r="H38" s="2" t="str">
-        <x:v>geo dm send 6vjvfv @anon4708 queued geo-dm-1785014611130 but history stayed empty; retry at real phone channel #etgcx requires explicit location-payload approval</x:v>
+        <x:v>geo dm send u4pruyd8 @anon4708 queued recheck_geo_dm_20260725 and persisted outbound state; post-fix history by nickname returned it; 814c9b6 adds regression coverage. Real #etgcx recipient delivery remains unconfirmed</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -2006,10 +2006,8 @@
           <x:t xml:space="preserve">src/bitchat_cli/app.py; src/bitchat_cli/queries.py; manual 2026-07-25</x:t>
         </x:is>
       </x:c>
-      <x:c r="H39" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">geo dm history 6vjvfv @trueanon --json executed with empty history</x:t>
-        </x:is>
+      <x:c r="H39" s="2" t="str">
+        <x:v>post-fix geo dm history u4pruyd8 @anon4708 --json returned the persisted recheck_geo_dm_20260725 outbound row</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -2900,8 +2898,7 @@
         </x:is>
       </x:c>
       <x:c r="B3" s="2" t="n">
-        <x:f>COUNTIF(Features!F2:F59,"Passed")</x:f>
-        <x:v>55</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="C3" s="2" t="inlineStr">
         <x:is>
@@ -2932,8 +2929,7 @@
         </x:is>
       </x:c>
       <x:c r="B5" s="2" t="n">
-        <x:f>COUNTIF(Features!F2:F59,"Blocked")</x:f>
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C5" s="2" t="inlineStr">
         <x:is>
@@ -2964,8 +2960,7 @@
         </x:is>
       </x:c>
       <x:c r="B7" s="4" t="n">
-        <x:f>IFERROR(B3/B2,0)</x:f>
-        <x:v>0.9482758620689655</x:v>
+        <x:v>0.9655172413793104</x:v>
       </x:c>
       <x:c r="C7" s="2" t="inlineStr">
         <x:is>
@@ -3035,15 +3030,11 @@
           <x:t xml:space="preserve">Current fix commit</x:t>
         </x:is>
       </x:c>
-      <x:c r="B12" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">20d5577</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C12" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Periodic BLE presence announcements</x:t>
-        </x:is>
+      <x:c r="B12" s="2" t="str">
+        <x:v>20d5577; 814c9b6</x:v>
+      </x:c>
+      <x:c r="C12" s="2" t="str">
+        <x:v>Periodic BLE presence announcements; geo-DM history resolves linked nicknames through Nostr identity</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3361,6 +3352,32 @@
         <x:v>Obtain explicit approval for the exact #etgcx payload, then verify receipt on Android and in the CLI history.</x:v>
       </x:c>
     </x:row>
+    <x:row r="9" ht="84" customHeight="1">
+      <x:c r="A9" s="6" t="str">
+        <x:v>ERR-008</x:v>
+      </x:c>
+      <x:c r="B9" s="6" t="str">
+        <x:v>2026-07-25</x:v>
+      </x:c>
+      <x:c r="C9" s="6" t="str">
+        <x:v>Geo DM history</x:v>
+      </x:c>
+      <x:c r="D9" s="6" t="str">
+        <x:v>A linked nickname resolved to the BitChat peer ID, while outbound geo-DM records are keyed by the participant's Nostr public key; history by nickname appeared empty after a successful queue.</x:v>
+      </x:c>
+      <x:c r="E9" s="6" t="str">
+        <x:v>Users could not inspect a geo-DM conversation by the nickname accepted by geo dm send.</x:v>
+      </x:c>
+      <x:c r="F9" s="6" t="str">
+        <x:v>Fixed</x:v>
+      </x:c>
+      <x:c r="G9" s="6" t="str">
+        <x:v>Manual u4pruyd8 test: history by @anon4708 returned empty, exact Nostr key returned recheck_geo_dm_20260725; 814c9b6; regression test in tests/test_app.py</x:v>
+      </x:c>
+      <x:c r="H9" s="6" t="str">
+        <x:v>Keep the nickname-to-Nostr-key regression test and verify history after future geo-DM sends.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: refresh regression count
</commit_message>
<xml_diff>
--- a/bitchat-cli-feature-tracker.xlsx
+++ b/bitchat-cli-feature-tracker.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="Rfeeaba20aa9e499a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Rac45f7e093e54f99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Errors" sheetId="3" r:id="Ra102cdb5d1554d79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="R3a3edad029114519"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R5804160bf55d46ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Errors" sheetId="3" r:id="Rc6f994e7d18b4421"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2583,7 +2583,7 @@
         </x:is>
       </x:c>
       <x:c r="H53" s="2" t="str">
-        <x:v>post-fix selftest ok; full pytest regression 177 passed</x:v>
+        <x:v>post-fix selftest ok; full pytest regression 178 passed</x:v>
       </x:c>
     </x:row>
     <x:row r="54">

</xml_diff>

<commit_message>
docs: record relay ack validation
</commit_message>
<xml_diff>
--- a/bitchat-cli-feature-tracker.xlsx
+++ b/bitchat-cli-feature-tracker.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="R3a3edad029114519"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R5804160bf55d46ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Errors" sheetId="3" r:id="Rc6f994e7d18b4421"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="R09602fe6a39f4121"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Rf5c9b51de5fa4a92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Errors" sheetId="3" r:id="R06206e05ddc94d73"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1383,7 +1383,7 @@
         </x:is>
       </x:c>
       <x:c r="F24" s="2" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="G24" s="2" t="inlineStr">
         <x:is>
@@ -1391,7 +1391,7 @@
         </x:is>
       </x:c>
       <x:c r="H24" s="2" t="str">
-        <x:v>geo send 6vjvfv remained blocked by relay HTTP 503; synthetic u4pruyd8 send recheck_geo_send_20260725 queued and was persisted, but no remote inbox confirmation was available</x:v>
+        <x:v>post-fix synthetic u4pruyd8 geo send ack_geo_send_final_20260725 completed after relay acknowledgement; 6vjvfv remains affected by a relay-specific HTTP 503</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -1967,7 +1967,7 @@
         </x:is>
       </x:c>
       <x:c r="H38" s="2" t="str">
-        <x:v>geo dm send u4pruyd8 @anon4708 queued recheck_geo_dm_20260725 and persisted outbound state; post-fix history by nickname returned it; 814c9b6 adds regression coverage. Real #etgcx recipient delivery remains unconfirmed</x:v>
+        <x:v>post-fix geo dm send u4pruyd8 @anon4708 ack_geo_dm_final_20260725 completed after relay acknowledgement; history by nickname returned the outbound row; real #etgcx recipient delivery remains unconfirmed</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -2583,7 +2583,7 @@
         </x:is>
       </x:c>
       <x:c r="H53" s="2" t="str">
-        <x:v>post-fix selftest ok; full pytest regression 178 passed</x:v>
+        <x:v>post-fix selftest ok; full pytest regression 180 passed</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -2898,7 +2898,7 @@
         </x:is>
       </x:c>
       <x:c r="B3" s="2" t="n">
-        <x:v>56</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="C3" s="2" t="inlineStr">
         <x:is>
@@ -2929,7 +2929,7 @@
         </x:is>
       </x:c>
       <x:c r="B5" s="2" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C5" s="2" t="inlineStr">
         <x:is>
@@ -2960,7 +2960,7 @@
         </x:is>
       </x:c>
       <x:c r="B7" s="4" t="n">
-        <x:v>0.9655172413793104</x:v>
+        <x:v>0.9827586206896551</x:v>
       </x:c>
       <x:c r="C7" s="2" t="inlineStr">
         <x:is>
@@ -3031,10 +3031,10 @@
         </x:is>
       </x:c>
       <x:c r="B12" s="2" t="str">
-        <x:v>20d5577; 814c9b6</x:v>
+        <x:v>20d5577; 814c9b6; 47eb720</x:v>
       </x:c>
       <x:c r="C12" s="2" t="str">
-        <x:v>Periodic BLE presence announcements; geo-DM history resolves linked nicknames through Nostr identity</x:v>
+        <x:v>Periodic BLE presence; geo-DM history identity resolution; relay publish acknowledgments</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3346,10 +3346,10 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="G8" s="6" t="str">
-        <x:v>geo dm send 6vjvfv @anon4708 manual_geo_dm_test_20260725; geo dm history 6vjvfv anon4708 --json returned []</x:v>
+        <x:v>Initial 6vjvfv geo dm had empty history; current u4pruyd8 ack_geo_dm_final_20260725 received relay acknowledgement and local history; real #etgcx recipient delivery remains unconfirmed</x:v>
       </x:c>
       <x:c r="H8" s="6" t="str">
-        <x:v>Obtain explicit approval for the exact #etgcx payload, then verify receipt on Android and in the CLI history.</x:v>
+        <x:v>Verify cross-device receipt on Android only after explicit approval for a real #etgcx payload.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="84" customHeight="1">
@@ -3376,6 +3376,32 @@
       </x:c>
       <x:c r="H9" s="6" t="str">
         <x:v>Keep the nickname-to-Nostr-key regression test and verify history after future geo-DM sends.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="84" customHeight="1">
+      <x:c r="A10" s="6" t="str">
+        <x:v>ERR-009</x:v>
+      </x:c>
+      <x:c r="B10" s="6" t="str">
+        <x:v>2026-07-25</x:v>
+      </x:c>
+      <x:c r="C10" s="6" t="str">
+        <x:v>Geochat/Nostr publish</x:v>
+      </x:c>
+      <x:c r="D10" s="6" t="str">
+        <x:v>The CLI reported a queued geohash or Nostr DM after sending a WebSocket EVENT, without waiting for the relay OK response; the message could be persisted while remote acceptance was unknown.</x:v>
+      </x:c>
+      <x:c r="E10" s="6" t="str">
+        <x:v>Users could mistake local persistence for relay delivery and investigate an empty remote inbox as if it were a recipient failure.</x:v>
+      </x:c>
+      <x:c r="F10" s="6" t="str">
+        <x:v>Fixed</x:v>
+      </x:c>
+      <x:c r="G10" s="6" t="str">
+        <x:v>Synthetic u4pruyd8 publish/inbox checks; 47eb720; tests/test_geochat.py and tests/test_nostr.py now cover OK=false rejection</x:v>
+      </x:c>
+      <x:c r="H10" s="6" t="str">
+        <x:v>Keep requiring a positive relay acknowledgement and treat partial relay failures as diagnostic evidence.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>